<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@a7c575853a252aec5f8c80387811fedd6f9f2bb9 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="246">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -121,114 +121,114 @@
     <t xml:space="preserve">Florida</t>
   </si>
   <si>
-    <t xml:space="preserve">PERODIAS DORIS_010252</t>
+    <t xml:space="preserve">Arauca_32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarragona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL REFUGIO 1, 2 Y 3_010139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chococito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INCAUCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Casilda_274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Pedregal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IND. DORIS_0453</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio de los Caballeros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTRAL CASTILLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA INDUSTRIA_752</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA CABAÑA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PISAMOS_0768</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REY 2_0784</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Diana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BELGICA_0780</t>
   </si>
   <si>
     <t xml:space="preserve">El Remolino</t>
   </si>
   <si>
-    <t xml:space="preserve">INCAUCA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-11-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arauca_32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarragona</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL REFUGIO 1, 2 Y 3_010139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chococito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Casilda_274</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Pedregal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IND. DORIS_0453</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Antonio de los Caballeros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CENTRAL CASTILLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA INDUSTRIA_752</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA CABAÑA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PISAMOS_0768</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REY 2_0784</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Diana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BELGICA_0780</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-04-30</t>
   </si>
   <si>
     <t xml:space="preserve">2026-06-16</t>
   </si>
   <si>
+    <t xml:space="preserve">LOS RANCHOS_0466</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-17</t>
+  </si>
+  <si>
     <t xml:space="preserve">Palmira</t>
   </si>
   <si>
@@ -328,415 +328,421 @@
     <t xml:space="preserve">2026-02-14</t>
   </si>
   <si>
-    <t xml:space="preserve">ING. NA</t>
+    <t xml:space="preserve">EL CUBO 1_0570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Granja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OTRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-03-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-06-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-04-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-09-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-09-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riesgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cofre_18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MITIGADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potrero de PA rraga_36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arenal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-09-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Arenal_48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA I_000204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARIA LUISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARGARITAS_0448</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Joaquin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabuyal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHONDULAR_940</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Palmar_88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA III_000207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cerrito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brisuelas_302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Helena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVACION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENOVA_2281</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL ALBION_080402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAJO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA HOLANDA_080355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMARIA_080104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Placer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-01-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL PLACER_080489</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURIN_080435</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-03-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFLEJO_305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-08-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROVIDENCIA_080101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-05-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA PAZ_080102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-07-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIERRA GRATA_0703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGENIO_000502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Retiro_384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA ESTRELLA_0725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Rosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAN RAFAEL H._0687</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Libano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WATERLOO_0484</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RIO FRAYLE_751</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERGOLA I_852</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PORVENIR_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boyaca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASCAJAL_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zamorano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAN JOSE_300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aguaclara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GERMANIA_367</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barrancas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GERTRUDIS_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amaime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASABCA/DOLORES_074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juanchito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPERANZA INESA_081363</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CABAA'A_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-10-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABROJAL_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-11-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SARITA_0434</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lomitas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL TABLON BAJO_B05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potrerito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA LEONA_0201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAYAPAN_0676</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONCORDIA_796</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARADO 2_0706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-07-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolo - Hartonal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MONASTIR_0436</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA FLORESTA_0761</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-08-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-22</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-03-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-06-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-04-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-09-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riesgo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cofre_18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MITIGADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potrero de PA rraga_36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arenal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Arenal_48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRITICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA I_000204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARIA LUISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARGARITAS_0448</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Joaquin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabuyal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHONDULAR_940</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Palmar_88</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA III_000207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-01-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cerrito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisuelas_302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Helena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GENOVA_2281</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Antonio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVACION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL ALBION_080402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BAJO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA HOLANDA_080355</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMARIA_080104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Placer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-01-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL PLACER_080489</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TURIN_080435</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-03-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFLEJO_305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-08-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROVIDENCIA_080101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-05-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA PAZ_080102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-07-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIERRA GRATA_0703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INGENIO_000502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Retiro_384</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA ESTRELLA_0725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Rosa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAN RAFAEL H._0687</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Libano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WATERLOO_0484</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RIO FRAYLE_751</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PERGOLA I_852</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORVENIR_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boyaca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASCAJAL_008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zamorano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAN JOSE_300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aguaclara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GERMANIA_367</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barrancas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GERTRUDIS_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amaime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASABCA/DOLORES_074</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juanchito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESPERANZA INESA_081363</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CABAA'A_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-10-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABROJAL_015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-11-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SARITA_0434</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lomitas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL TABLON BAJO_B05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potrerito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA LEONA_0201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAYAPAN_0676</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Granja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONCORDIA_796</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARADO 2_0706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-07-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bolo - Hartonal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MONASTIR_0436</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA FLORESTA_0761</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-08-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-22</t>
   </si>
   <si>
     <t xml:space="preserve">2026-01-25</t>
@@ -1277,16 +1283,16 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
         <v>37</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
-        <v>39</v>
-      </c>
       <c r="G7" t="n">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
@@ -1303,13 +1309,13 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
         <v>40</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
       </c>
       <c r="E8" t="s">
         <v>42</v>
@@ -1318,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="G8" t="n">
-        <v>98</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
         <v>16</v>
@@ -1341,7 +1347,7 @@
         <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
         <v>46</v>
@@ -1350,7 +1356,7 @@
         <v>47</v>
       </c>
       <c r="G9" t="n">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
@@ -1373,16 +1379,16 @@
         <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -1399,10 +1405,10 @@
         <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
         <v>54</v>
@@ -1414,7 +1420,7 @@
         <v>56</v>
       </c>
       <c r="G11" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -1434,19 +1440,19 @@
         <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
         <v>58</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>59</v>
       </c>
-      <c r="F12" t="s">
-        <v>60</v>
-      </c>
       <c r="G12" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -1463,13 +1469,13 @@
         <v>34</v>
       </c>
       <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s">
         <v>61</v>
       </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
         <v>62</v>
@@ -1478,7 +1484,7 @@
         <v>63</v>
       </c>
       <c r="G13" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -1501,7 +1507,7 @@
         <v>65</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
         <v>66</v>
@@ -1510,7 +1516,7 @@
         <v>67</v>
       </c>
       <c r="G14" t="n">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -1530,10 +1536,10 @@
         <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
         <v>69</v>
@@ -1542,7 +1548,7 @@
         <v>70</v>
       </c>
       <c r="G15" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -1571,7 +1577,7 @@
         <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G16" t="n">
         <v>10</v>
@@ -1597,7 +1603,7 @@
         <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
         <v>77</v>
@@ -1635,7 +1641,7 @@
         <v>82</v>
       </c>
       <c r="F18" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G18" t="n">
         <v>34</v>
@@ -1696,10 +1702,10 @@
         <v>28</v>
       </c>
       <c r="E20" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G20" t="n">
         <v>57</v>
@@ -1795,7 +1801,7 @@
         <v>100</v>
       </c>
       <c r="F23" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G23" t="n">
         <v>47</v>
@@ -1827,36 +1833,42 @@
         <v>103</v>
       </c>
       <c r="F24" t="s">
+        <v>67</v>
+      </c>
+      <c r="G24" t="n">
+        <v>16</v>
+      </c>
+      <c r="H24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" t="s">
         <v>70</v>
       </c>
-      <c r="G24" t="n">
-        <v>16</v>
-      </c>
-      <c r="H24" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" t="s">
-        <v>17</v>
-      </c>
-      <c r="J24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25"/>
-      <c r="D25" t="s">
-        <v>104</v>
-      </c>
-      <c r="E25" t="s">
-        <v>105</v>
-      </c>
-      <c r="F25" t="s">
-        <v>39</v>
-      </c>
       <c r="G25" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="H25" t="s">
         <v>16</v>
@@ -1873,13 +1885,13 @@
       <c r="B26"/>
       <c r="C26"/>
       <c r="D26" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E26" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F26" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G26" t="n">
         <v>6</v>
@@ -1899,13 +1911,13 @@
       <c r="B27"/>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F27" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G27" t="n">
         <v>4</v>
@@ -1925,13 +1937,13 @@
       <c r="B28"/>
       <c r="C28"/>
       <c r="D28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F28" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G28" t="n">
         <v>2</v>
@@ -1951,13 +1963,13 @@
       <c r="B29"/>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G29" t="n">
         <v>7</v>
@@ -1977,13 +1989,13 @@
       <c r="B30"/>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E30" t="s">
         <v>82</v>
       </c>
       <c r="F30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G30" t="n">
         <v>49</v>
@@ -2003,13 +2015,13 @@
       <c r="B31"/>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G31" t="n">
         <v>9</v>
@@ -2029,13 +2041,13 @@
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G32" t="n">
         <v>3</v>
@@ -2055,13 +2067,13 @@
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F33" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G33" t="n">
         <v>9</v>
@@ -2081,13 +2093,13 @@
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G34" t="n">
         <v>6</v>
@@ -2107,10 +2119,10 @@
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E35" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F35" t="s">
         <v>87</v>
@@ -2133,10 +2145,10 @@
       <c r="B36"/>
       <c r="C36"/>
       <c r="D36" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E36" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F36" t="s">
         <v>87</v>
@@ -2159,13 +2171,13 @@
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E37" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F37" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G37" t="n">
         <v>20</v>
@@ -2185,13 +2197,13 @@
       <c r="B38"/>
       <c r="C38"/>
       <c r="D38" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E38" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F38" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G38" t="n">
         <v>8</v>
@@ -2211,10 +2223,10 @@
       <c r="B39"/>
       <c r="C39"/>
       <c r="D39" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E39" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F39" t="s">
         <v>33</v>
@@ -2237,10 +2249,10 @@
       <c r="B40"/>
       <c r="C40"/>
       <c r="D40" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E40" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F40" t="s">
         <v>33</v>
@@ -2263,10 +2275,10 @@
       <c r="B41"/>
       <c r="C41"/>
       <c r="D41" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E41" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F41" t="s">
         <v>33</v>
@@ -2289,13 +2301,13 @@
       <c r="B42"/>
       <c r="C42"/>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E42" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F42" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G42" t="n">
         <v>41</v>
@@ -2315,13 +2327,13 @@
       <c r="B43"/>
       <c r="C43"/>
       <c r="D43" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E43" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F43" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G43" t="n">
         <v>39</v>
@@ -2341,13 +2353,13 @@
       <c r="B44"/>
       <c r="C44"/>
       <c r="D44" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E44" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F44" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G44" t="n">
         <v>5</v>
@@ -2367,7 +2379,7 @@
       <c r="B45"/>
       <c r="C45"/>
       <c r="D45" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E45" t="s">
         <v>77</v>
@@ -2393,7 +2405,7 @@
       <c r="B46"/>
       <c r="C46"/>
       <c r="D46" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E46" t="s">
         <v>14</v>
@@ -2419,13 +2431,13 @@
       <c r="B47"/>
       <c r="C47"/>
       <c r="D47" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E47" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F47" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G47" t="n">
         <v>8</v>
@@ -2445,13 +2457,13 @@
       <c r="B48"/>
       <c r="C48"/>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E48" t="s">
         <v>82</v>
       </c>
       <c r="F48" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G48" t="n">
         <v>10</v>
@@ -2471,13 +2483,13 @@
       <c r="B49"/>
       <c r="C49"/>
       <c r="D49" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E49" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F49" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G49" t="n">
         <v>2</v>
@@ -2497,13 +2509,13 @@
       <c r="B50"/>
       <c r="C50"/>
       <c r="D50" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E50" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F50" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G50" t="n">
         <v>17</v>
@@ -2543,7 +2555,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -2566,7 +2578,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -2575,10 +2587,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G2" t="n">
         <v>74</v>
@@ -2598,19 +2610,19 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G3" t="n">
         <v>70</v>
@@ -2630,19 +2642,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" t="s">
         <v>142</v>
-      </c>
-      <c r="C4" t="s">
-        <v>140</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -2662,19 +2674,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G5" t="n">
         <v>63</v>
@@ -2694,19 +2706,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
@@ -2726,19 +2738,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G7" t="n">
         <v>59</v>
@@ -2758,19 +2770,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" t="s">
         <v>154</v>
       </c>
-      <c r="C8" t="s">
-        <v>152</v>
-      </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G8" t="n">
         <v>58</v>
@@ -2790,7 +2802,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2799,10 +2811,10 @@
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G9" t="n">
         <v>46</v>
@@ -2822,7 +2834,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
@@ -2831,10 +2843,10 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G10" t="n">
         <v>45</v>
@@ -2854,19 +2866,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G11" t="n">
         <v>34</v>
@@ -2883,22 +2895,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G12" t="n">
         <v>62</v>
@@ -2915,22 +2927,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B13" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D13" t="s">
         <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -2947,19 +2959,19 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
         <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F14" t="s">
         <v>86</v>
@@ -2979,22 +2991,22 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C15" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
         <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F15" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G15" t="n">
         <v>7</v>
@@ -3011,22 +3023,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D16" t="s">
         <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G16" t="n">
         <v>6</v>
@@ -3043,22 +3055,22 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B17" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D17" t="s">
         <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F17" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -3075,22 +3087,22 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C18" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D18" t="s">
         <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -3107,22 +3119,22 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -3139,22 +3151,22 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B20" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D20" t="s">
         <v>85</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -3171,22 +3183,22 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B21" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D21" t="s">
         <v>85</v>
       </c>
       <c r="E21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F21" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -3206,19 +3218,19 @@
         <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F22" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G22" t="n">
         <v>154</v>
@@ -3238,19 +3250,19 @@
         <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G23" t="n">
         <v>144</v>
@@ -3270,16 +3282,16 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C24" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D24" t="s">
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
@@ -3302,19 +3314,19 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C25" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D25" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F25" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G25" t="n">
         <v>100</v>
@@ -3334,19 +3346,19 @@
         <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D26" t="s">
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F26" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G26" t="n">
         <v>98</v>
@@ -3366,19 +3378,19 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C27" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D27" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E27" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F27" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G27" t="n">
         <v>82</v>
@@ -3398,19 +3410,19 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F28" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G28" t="n">
         <v>79</v>
@@ -3430,19 +3442,19 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E29" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F29" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G29" t="n">
         <v>67</v>
@@ -3462,19 +3474,19 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C30" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D30" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E30" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F30" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G30" t="n">
         <v>63</v>
@@ -3494,19 +3506,19 @@
         <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C31" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E31" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F31" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G31" t="n">
         <v>63</v>
@@ -3526,19 +3538,19 @@
         <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C32" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F32" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G32" t="n">
         <v>156</v>
@@ -3558,16 +3570,16 @@
         <v>71</v>
       </c>
       <c r="B33" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C33" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F33" t="s">
         <v>82</v>
@@ -3590,19 +3602,19 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C34" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G34" t="n">
         <v>118</v>
@@ -3622,16 +3634,16 @@
         <v>71</v>
       </c>
       <c r="B35" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C35" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F35" t="s">
         <v>92</v>
@@ -3654,19 +3666,19 @@
         <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C36" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F36" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G36" t="n">
         <v>112</v>
@@ -3686,19 +3698,19 @@
         <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C37" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F37" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G37" t="n">
         <v>106</v>
@@ -3718,7 +3730,7 @@
         <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C38" t="s">
         <v>91</v>
@@ -3727,10 +3739,10 @@
         <v>85</v>
       </c>
       <c r="E38" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G38" t="n">
         <v>101</v>
@@ -3750,7 +3762,7 @@
         <v>71</v>
       </c>
       <c r="B39" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C39" t="s">
         <v>89</v>
@@ -3759,10 +3771,10 @@
         <v>28</v>
       </c>
       <c r="E39" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F39" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G39" t="n">
         <v>98</v>
@@ -3782,7 +3794,7 @@
         <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C40" t="s">
         <v>94</v>
@@ -3791,10 +3803,10 @@
         <v>28</v>
       </c>
       <c r="E40" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F40" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G40" t="n">
         <v>68</v>
@@ -3823,10 +3835,10 @@
         <v>28</v>
       </c>
       <c r="E41" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F41" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G41" t="n">
         <v>57</v>
@@ -3846,16 +3858,16 @@
         <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C42" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D42" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E42" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3878,19 +3890,19 @@
         <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C43" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D43" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E43" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F43" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G43" t="n">
         <v>48</v>
@@ -3919,7 +3931,7 @@
         <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F44" t="s">
         <v>100</v>
@@ -3942,19 +3954,19 @@
         <v>97</v>
       </c>
       <c r="B45" t="s">
+        <v>227</v>
+      </c>
+      <c r="C45" t="s">
         <v>225</v>
       </c>
-      <c r="C45" t="s">
-        <v>223</v>
-      </c>
       <c r="D45" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E45" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F45" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G45" t="n">
         <v>39</v>
@@ -3974,19 +3986,19 @@
         <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C46" t="s">
-        <v>228</v>
+        <v>105</v>
       </c>
       <c r="D46" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E46" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F46" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G46" t="n">
         <v>31</v>
@@ -4006,7 +4018,7 @@
         <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C47" t="s">
         <v>99</v>
@@ -4015,7 +4027,7 @@
         <v>28</v>
       </c>
       <c r="E47" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F47" t="s">
         <v>86</v>
@@ -4038,19 +4050,19 @@
         <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C48" t="s">
         <v>99</v>
       </c>
       <c r="D48" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E48" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F48" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G48" t="n">
         <v>27</v>
@@ -4070,19 +4082,19 @@
         <v>97</v>
       </c>
       <c r="B49" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C49" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D49" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E49" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F49" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -4102,19 +4114,19 @@
         <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C50" t="s">
-        <v>228</v>
+        <v>105</v>
       </c>
       <c r="D50" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E50" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G50" t="n">
         <v>24</v>
@@ -4134,19 +4146,19 @@
         <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C51" t="s">
         <v>99</v>
       </c>
       <c r="D51" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E51" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F51" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G51" t="n">
         <v>21</v>
@@ -4166,10 +4178,10 @@
       <c r="B52"/>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E52" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F52" t="s">
         <v>82</v>
@@ -4192,13 +4204,13 @@
       <c r="B53"/>
       <c r="C53"/>
       <c r="D53" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E53" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F53" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G53" t="n">
         <v>127</v>
@@ -4218,13 +4230,13 @@
       <c r="B54"/>
       <c r="C54"/>
       <c r="D54" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E54" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F54" t="s">
-        <v>105</v>
+        <v>242</v>
       </c>
       <c r="G54" t="n">
         <v>74</v>
@@ -4244,13 +4256,13 @@
       <c r="B55"/>
       <c r="C55"/>
       <c r="D55" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E55" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F55" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G55" t="n">
         <v>74</v>
@@ -4270,13 +4282,13 @@
       <c r="B56"/>
       <c r="C56"/>
       <c r="D56" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E56" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F56" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G56" t="n">
         <v>59</v>
@@ -4296,13 +4308,13 @@
       <c r="B57"/>
       <c r="C57"/>
       <c r="D57" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E57" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F57" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G57" t="n">
         <v>53</v>
@@ -4322,10 +4334,10 @@
       <c r="B58"/>
       <c r="C58"/>
       <c r="D58" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E58" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F58" t="s">
         <v>82</v>
@@ -4348,13 +4360,13 @@
       <c r="B59"/>
       <c r="C59"/>
       <c r="D59" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E59" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F59" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G59" t="n">
         <v>48</v>
@@ -4374,10 +4386,10 @@
       <c r="B60"/>
       <c r="C60"/>
       <c r="D60" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E60" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F60" t="s">
         <v>92</v>
@@ -4400,13 +4412,13 @@
       <c r="B61"/>
       <c r="C61"/>
       <c r="D61" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E61" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F61" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G61" t="n">
         <v>43</v>
@@ -4446,7 +4458,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -4469,10 +4481,10 @@
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F2" t="s">
         <v>82</v>
@@ -4495,19 +4507,19 @@
         <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G3" t="n">
         <v>156</v>
@@ -4527,19 +4539,19 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>154</v>
@@ -4559,19 +4571,19 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G5" t="n">
         <v>144</v>
@@ -4591,13 +4603,13 @@
       <c r="B6"/>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G6" t="n">
         <v>127</v>
@@ -4617,16 +4629,16 @@
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C7" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="F7" t="s">
         <v>82</v>
@@ -4649,16 +4661,16 @@
         <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F8" t="s">
         <v>92</v>
@@ -4681,19 +4693,19 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G9" t="n">
         <v>118</v>
@@ -4713,16 +4725,16 @@
         <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F10" t="s">
         <v>92</v>
@@ -4745,19 +4757,19 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
       </c>
       <c r="E11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G11" t="n">
         <v>112</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@9de9a55f745e5956328dda292df924d50d5f299a 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -337,282 +337,195 @@
     <t xml:space="preserve">2025-12-20</t>
   </si>
   <si>
-    <t xml:space="preserve">OTRO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-03-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-06-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-04-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-09-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-23</t>
+    <t xml:space="preserve">Riesgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cofre_18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MITIGADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potrero de PA rraga_36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arenal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-09-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Arenal_48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA I_000204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARIA LUISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARGARITAS_0448</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Joaquin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabuyal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHONDULAR_940</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Palmar_88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA III_000207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cerrito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brisuelas_302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Helena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVACION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENOVA_2281</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL ALBION_080402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAJO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA HOLANDA_080355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMARIA_080104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Placer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-01-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL PLACER_080489</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURIN_080435</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-03-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFLEJO_305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-08-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROVIDENCIA_080101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-05-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA PAZ_080102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-07-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIERRA GRATA_0703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGENIO_000502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Retiro_384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA ESTRELLA_0725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Rosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAN RAFAEL H._0687</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Libano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WATERLOO_0484</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RIO FRAYLE_751</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-08</t>
   </si>
   <si>
-    <t xml:space="preserve">2025-09-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riesgo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cofre_18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MITIGADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potrero de PA rraga_36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arenal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Arenal_48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRITICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA I_000204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARIA LUISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARGARITAS_0448</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Joaquin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabuyal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHONDULAR_940</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Palmar_88</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA III_000207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-01-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cerrito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisuelas_302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Helena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVACION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GENOVA_2281</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Antonio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL ALBION_080402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BAJO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA HOLANDA_080355</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMARIA_080104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Placer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-01-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL PLACER_080489</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TURIN_080435</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-03-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFLEJO_305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-08-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROVIDENCIA_080101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-05-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA PAZ_080102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-07-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIERRA GRATA_0703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INGENIO_000502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Retiro_384</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA ESTRELLA_0725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Rosa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAN RAFAEL H._0687</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Libano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WATERLOO_0484</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RIO FRAYLE_751</t>
-  </si>
-  <si>
     <t xml:space="preserve">PERGOLA I_852</t>
   </si>
   <si>
@@ -739,16 +652,25 @@
     <t xml:space="preserve">2023-08-04</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-31</t>
+    <t xml:space="preserve">LA MERCED CABAL HNAS._080500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022-09-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA CLARA_0637</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019-09-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA PACHITA_010749</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin Eventos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita Preventiva</t>
   </si>
   <si>
     <t xml:space="preserve">Nivel</t>
@@ -1880,656 +1802,6 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26"/>
-      <c r="B26"/>
-      <c r="C26"/>
-      <c r="D26" t="s">
-        <v>107</v>
-      </c>
-      <c r="E26" t="s">
-        <v>108</v>
-      </c>
-      <c r="F26" t="s">
-        <v>109</v>
-      </c>
-      <c r="G26" t="n">
-        <v>6</v>
-      </c>
-      <c r="H26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" t="s">
-        <v>17</v>
-      </c>
-      <c r="J26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27"/>
-      <c r="B27"/>
-      <c r="C27"/>
-      <c r="D27" t="s">
-        <v>107</v>
-      </c>
-      <c r="E27" t="s">
-        <v>110</v>
-      </c>
-      <c r="F27" t="s">
-        <v>109</v>
-      </c>
-      <c r="G27" t="n">
-        <v>4</v>
-      </c>
-      <c r="H27" t="s">
-        <v>16</v>
-      </c>
-      <c r="I27" t="s">
-        <v>17</v>
-      </c>
-      <c r="J27" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28"/>
-      <c r="B28"/>
-      <c r="C28"/>
-      <c r="D28" t="s">
-        <v>107</v>
-      </c>
-      <c r="E28" t="s">
-        <v>111</v>
-      </c>
-      <c r="F28" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" t="s">
-        <v>17</v>
-      </c>
-      <c r="J28" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29" t="s">
-        <v>107</v>
-      </c>
-      <c r="E29" t="s">
-        <v>112</v>
-      </c>
-      <c r="F29" t="s">
-        <v>43</v>
-      </c>
-      <c r="G29" t="n">
-        <v>7</v>
-      </c>
-      <c r="H29" t="s">
-        <v>16</v>
-      </c>
-      <c r="I29" t="s">
-        <v>17</v>
-      </c>
-      <c r="J29" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30" t="s">
-        <v>107</v>
-      </c>
-      <c r="E30" t="s">
-        <v>82</v>
-      </c>
-      <c r="F30" t="s">
-        <v>113</v>
-      </c>
-      <c r="G30" t="n">
-        <v>49</v>
-      </c>
-      <c r="H30" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" t="s">
-        <v>17</v>
-      </c>
-      <c r="J30" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31" t="s">
-        <v>107</v>
-      </c>
-      <c r="E31" t="s">
-        <v>114</v>
-      </c>
-      <c r="F31" t="s">
-        <v>115</v>
-      </c>
-      <c r="G31" t="n">
-        <v>9</v>
-      </c>
-      <c r="H31" t="s">
-        <v>16</v>
-      </c>
-      <c r="I31" t="s">
-        <v>17</v>
-      </c>
-      <c r="J31" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32" t="s">
-        <v>107</v>
-      </c>
-      <c r="E32" t="s">
-        <v>116</v>
-      </c>
-      <c r="F32" t="s">
-        <v>115</v>
-      </c>
-      <c r="G32" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" t="s">
-        <v>17</v>
-      </c>
-      <c r="J32" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33" t="s">
-        <v>107</v>
-      </c>
-      <c r="E33" t="s">
-        <v>117</v>
-      </c>
-      <c r="F33" t="s">
-        <v>47</v>
-      </c>
-      <c r="G33" t="n">
-        <v>9</v>
-      </c>
-      <c r="H33" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" t="s">
-        <v>17</v>
-      </c>
-      <c r="J33" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
-      <c r="D34" t="s">
-        <v>107</v>
-      </c>
-      <c r="E34" t="s">
-        <v>118</v>
-      </c>
-      <c r="F34" t="s">
-        <v>119</v>
-      </c>
-      <c r="G34" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" t="s">
-        <v>17</v>
-      </c>
-      <c r="J34" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35" t="s">
-        <v>107</v>
-      </c>
-      <c r="E35" t="s">
-        <v>120</v>
-      </c>
-      <c r="F35" t="s">
-        <v>87</v>
-      </c>
-      <c r="G35" t="n">
-        <v>4</v>
-      </c>
-      <c r="H35" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35" t="s">
-        <v>17</v>
-      </c>
-      <c r="J35" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36" t="s">
-        <v>107</v>
-      </c>
-      <c r="E36" t="s">
-        <v>121</v>
-      </c>
-      <c r="F36" t="s">
-        <v>87</v>
-      </c>
-      <c r="G36" t="n">
-        <v>4</v>
-      </c>
-      <c r="H36" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" t="s">
-        <v>17</v>
-      </c>
-      <c r="J36" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" t="s">
-        <v>122</v>
-      </c>
-      <c r="F37" t="s">
-        <v>123</v>
-      </c>
-      <c r="G37" t="n">
-        <v>20</v>
-      </c>
-      <c r="H37" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" t="s">
-        <v>17</v>
-      </c>
-      <c r="J37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38"/>
-      <c r="B38"/>
-      <c r="C38"/>
-      <c r="D38" t="s">
-        <v>107</v>
-      </c>
-      <c r="E38" t="s">
-        <v>124</v>
-      </c>
-      <c r="F38" t="s">
-        <v>125</v>
-      </c>
-      <c r="G38" t="n">
-        <v>8</v>
-      </c>
-      <c r="H38" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" t="s">
-        <v>17</v>
-      </c>
-      <c r="J38" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39" t="s">
-        <v>107</v>
-      </c>
-      <c r="E39" t="s">
-        <v>126</v>
-      </c>
-      <c r="F39" t="s">
-        <v>33</v>
-      </c>
-      <c r="G39" t="n">
-        <v>33</v>
-      </c>
-      <c r="H39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s">
-        <v>17</v>
-      </c>
-      <c r="J39" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40" t="s">
-        <v>107</v>
-      </c>
-      <c r="E40" t="s">
-        <v>127</v>
-      </c>
-      <c r="F40" t="s">
-        <v>33</v>
-      </c>
-      <c r="G40" t="n">
-        <v>15</v>
-      </c>
-      <c r="H40" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40" t="s">
-        <v>17</v>
-      </c>
-      <c r="J40" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41"/>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41" t="s">
-        <v>107</v>
-      </c>
-      <c r="E41" t="s">
-        <v>128</v>
-      </c>
-      <c r="F41" t="s">
-        <v>33</v>
-      </c>
-      <c r="G41" t="n">
-        <v>9</v>
-      </c>
-      <c r="H41" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" t="s">
-        <v>17</v>
-      </c>
-      <c r="J41" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42"/>
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42" t="s">
-        <v>107</v>
-      </c>
-      <c r="E42" t="s">
-        <v>129</v>
-      </c>
-      <c r="F42" t="s">
-        <v>59</v>
-      </c>
-      <c r="G42" t="n">
-        <v>41</v>
-      </c>
-      <c r="H42" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" t="s">
-        <v>17</v>
-      </c>
-      <c r="J42" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43"/>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43" t="s">
-        <v>107</v>
-      </c>
-      <c r="E43" t="s">
-        <v>130</v>
-      </c>
-      <c r="F43" t="s">
-        <v>59</v>
-      </c>
-      <c r="G43" t="n">
-        <v>39</v>
-      </c>
-      <c r="H43" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" t="s">
-        <v>17</v>
-      </c>
-      <c r="J43" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44"/>
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44" t="s">
-        <v>107</v>
-      </c>
-      <c r="E44" t="s">
-        <v>131</v>
-      </c>
-      <c r="F44" t="s">
-        <v>132</v>
-      </c>
-      <c r="G44" t="n">
-        <v>5</v>
-      </c>
-      <c r="H44" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" t="s">
-        <v>17</v>
-      </c>
-      <c r="J44" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45"/>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45" t="s">
-        <v>107</v>
-      </c>
-      <c r="E45" t="s">
-        <v>77</v>
-      </c>
-      <c r="F45" t="s">
-        <v>96</v>
-      </c>
-      <c r="G45" t="n">
-        <v>35</v>
-      </c>
-      <c r="H45" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" t="s">
-        <v>17</v>
-      </c>
-      <c r="J45" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46" t="s">
-        <v>107</v>
-      </c>
-      <c r="E46" t="s">
-        <v>14</v>
-      </c>
-      <c r="F46" t="s">
-        <v>96</v>
-      </c>
-      <c r="G46" t="n">
-        <v>2</v>
-      </c>
-      <c r="H46" t="s">
-        <v>16</v>
-      </c>
-      <c r="I46" t="s">
-        <v>17</v>
-      </c>
-      <c r="J46" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47"/>
-      <c r="B47"/>
-      <c r="C47"/>
-      <c r="D47" t="s">
-        <v>107</v>
-      </c>
-      <c r="E47" t="s">
-        <v>133</v>
-      </c>
-      <c r="F47" t="s">
-        <v>134</v>
-      </c>
-      <c r="G47" t="n">
-        <v>8</v>
-      </c>
-      <c r="H47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" t="s">
-        <v>17</v>
-      </c>
-      <c r="J47" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48"/>
-      <c r="B48"/>
-      <c r="C48"/>
-      <c r="D48" t="s">
-        <v>107</v>
-      </c>
-      <c r="E48" t="s">
-        <v>82</v>
-      </c>
-      <c r="F48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G48" t="n">
-        <v>10</v>
-      </c>
-      <c r="H48" t="s">
-        <v>16</v>
-      </c>
-      <c r="I48" t="s">
-        <v>17</v>
-      </c>
-      <c r="J48" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49"/>
-      <c r="B49"/>
-      <c r="C49"/>
-      <c r="D49" t="s">
-        <v>107</v>
-      </c>
-      <c r="E49" t="s">
-        <v>135</v>
-      </c>
-      <c r="F49" t="s">
-        <v>67</v>
-      </c>
-      <c r="G49" t="n">
-        <v>2</v>
-      </c>
-      <c r="H49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" t="s">
-        <v>17</v>
-      </c>
-      <c r="J49" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50"/>
-      <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50" t="s">
-        <v>107</v>
-      </c>
-      <c r="E50" t="s">
-        <v>136</v>
-      </c>
-      <c r="F50" t="s">
-        <v>67</v>
-      </c>
-      <c r="G50" t="n">
-        <v>17</v>
-      </c>
-      <c r="H50" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" t="s">
-        <v>17</v>
-      </c>
-      <c r="J50" t="s">
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -2555,7 +1827,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -2578,7 +1850,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>108</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -2587,10 +1859,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F2" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G2" t="n">
         <v>74</v>
@@ -2610,19 +1882,19 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="G3" t="n">
         <v>70</v>
@@ -2642,19 +1914,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F4" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -2674,19 +1946,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F5" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
       <c r="G5" t="n">
         <v>63</v>
@@ -2706,19 +1978,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
         <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
@@ -2738,19 +2010,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="C7" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="D7" t="s">
         <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F7" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="G7" t="n">
         <v>59</v>
@@ -2770,19 +2042,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="D8" t="s">
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F8" t="s">
-        <v>157</v>
+        <v>127</v>
       </c>
       <c r="G8" t="n">
         <v>58</v>
@@ -2802,7 +2074,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2811,10 +2083,10 @@
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F9" t="s">
-        <v>159</v>
+        <v>129</v>
       </c>
       <c r="G9" t="n">
         <v>46</v>
@@ -2834,7 +2106,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>160</v>
+        <v>130</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
@@ -2843,7 +2115,7 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F10" t="s">
         <v>37</v>
@@ -2866,19 +2138,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E11" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F11" t="s">
-        <v>162</v>
+        <v>132</v>
       </c>
       <c r="G11" t="n">
         <v>34</v>
@@ -2895,22 +2167,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B12" t="s">
-        <v>164</v>
+        <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>165</v>
+        <v>135</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="F12" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
       <c r="G12" t="n">
         <v>62</v>
@@ -2927,22 +2199,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B13" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D13" t="s">
         <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="F13" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -2959,19 +2231,19 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
       <c r="C14" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D14" t="s">
         <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="F14" t="s">
         <v>86</v>
@@ -2991,19 +2263,19 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B15" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
       <c r="C15" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D15" t="s">
         <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="F15" t="s">
         <v>37</v>
@@ -3023,22 +2295,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B16" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="D16" t="s">
         <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F16" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="G16" t="n">
         <v>6</v>
@@ -3055,22 +2327,22 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B17" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="D17" t="s">
         <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F17" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -3087,22 +2359,22 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B18" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D18" t="s">
         <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F18" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -3119,22 +2391,22 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B19" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="C19" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F19" t="s">
-        <v>182</v>
+        <v>152</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -3151,22 +2423,22 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B20" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
       <c r="C20" t="s">
-        <v>165</v>
+        <v>135</v>
       </c>
       <c r="D20" t="s">
         <v>85</v>
       </c>
       <c r="E20" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F20" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -3183,22 +2455,22 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="B21" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="C21" t="s">
-        <v>165</v>
+        <v>135</v>
       </c>
       <c r="D21" t="s">
         <v>85</v>
       </c>
       <c r="E21" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F21" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -3218,7 +2490,7 @@
         <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
@@ -3227,7 +2499,7 @@
         <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
         <v>37</v>
@@ -3250,19 +2522,19 @@
         <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="C23" t="s">
         <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F23" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="G23" t="n">
         <v>144</v>
@@ -3282,7 +2554,7 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="C24" t="s">
         <v>65</v>
@@ -3291,7 +2563,7 @@
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
@@ -3314,19 +2586,19 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>191</v>
+        <v>161</v>
       </c>
       <c r="C25" t="s">
-        <v>192</v>
+        <v>162</v>
       </c>
       <c r="D25" t="s">
         <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F25" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G25" t="n">
         <v>100</v>
@@ -3355,7 +2627,7 @@
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F26" t="s">
         <v>37</v>
@@ -3378,16 +2650,16 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
       <c r="D27" t="s">
         <v>50</v>
       </c>
       <c r="E27" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
         <v>58</v>
@@ -3419,7 +2691,7 @@
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F28" t="s">
         <v>46</v>
@@ -3442,7 +2714,7 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>196</v>
+        <v>166</v>
       </c>
       <c r="C29" t="s">
         <v>61</v>
@@ -3451,10 +2723,10 @@
         <v>50</v>
       </c>
       <c r="E29" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="F29" t="s">
-        <v>197</v>
+        <v>167</v>
       </c>
       <c r="G29" t="n">
         <v>67</v>
@@ -3474,7 +2746,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>198</v>
+        <v>168</v>
       </c>
       <c r="C30" t="s">
         <v>65</v>
@@ -3483,10 +2755,10 @@
         <v>54</v>
       </c>
       <c r="E30" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F30" t="s">
-        <v>130</v>
+        <v>169</v>
       </c>
       <c r="G30" t="n">
         <v>63</v>
@@ -3506,7 +2778,7 @@
         <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="C31" t="s">
         <v>61</v>
@@ -3515,10 +2787,10 @@
         <v>54</v>
       </c>
       <c r="E31" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F31" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="G31" t="n">
         <v>63</v>
@@ -3538,19 +2810,19 @@
         <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>201</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>202</v>
+        <v>173</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F32" t="s">
-        <v>203</v>
+        <v>174</v>
       </c>
       <c r="G32" t="n">
         <v>156</v>
@@ -3570,16 +2842,16 @@
         <v>71</v>
       </c>
       <c r="B33" t="s">
-        <v>204</v>
+        <v>175</v>
       </c>
       <c r="C33" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F33" t="s">
         <v>82</v>
@@ -3602,19 +2874,19 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="C34" t="s">
-        <v>207</v>
+        <v>178</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
-        <v>208</v>
+        <v>179</v>
       </c>
       <c r="G34" t="n">
         <v>118</v>
@@ -3634,16 +2906,16 @@
         <v>71</v>
       </c>
       <c r="B35" t="s">
-        <v>209</v>
+        <v>180</v>
       </c>
       <c r="C35" t="s">
-        <v>210</v>
+        <v>181</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F35" t="s">
         <v>92</v>
@@ -3666,19 +2938,19 @@
         <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>211</v>
+        <v>182</v>
       </c>
       <c r="C36" t="s">
-        <v>212</v>
+        <v>183</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F36" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G36" t="n">
         <v>112</v>
@@ -3698,19 +2970,19 @@
         <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
-        <v>214</v>
+        <v>185</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F37" t="s">
-        <v>215</v>
+        <v>186</v>
       </c>
       <c r="G37" t="n">
         <v>106</v>
@@ -3730,7 +3002,7 @@
         <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>216</v>
+        <v>187</v>
       </c>
       <c r="C38" t="s">
         <v>91</v>
@@ -3739,10 +3011,10 @@
         <v>85</v>
       </c>
       <c r="E38" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F38" t="s">
-        <v>217</v>
+        <v>188</v>
       </c>
       <c r="G38" t="n">
         <v>101</v>
@@ -3762,7 +3034,7 @@
         <v>71</v>
       </c>
       <c r="B39" t="s">
-        <v>218</v>
+        <v>189</v>
       </c>
       <c r="C39" t="s">
         <v>89</v>
@@ -3771,10 +3043,10 @@
         <v>28</v>
       </c>
       <c r="E39" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F39" t="s">
-        <v>219</v>
+        <v>190</v>
       </c>
       <c r="G39" t="n">
         <v>98</v>
@@ -3794,7 +3066,7 @@
         <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>220</v>
+        <v>191</v>
       </c>
       <c r="C40" t="s">
         <v>94</v>
@@ -3803,10 +3075,10 @@
         <v>28</v>
       </c>
       <c r="E40" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F40" t="s">
-        <v>221</v>
+        <v>192</v>
       </c>
       <c r="G40" t="n">
         <v>68</v>
@@ -3835,7 +3107,7 @@
         <v>28</v>
       </c>
       <c r="E41" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F41" t="s">
         <v>37</v>
@@ -3858,16 +3130,16 @@
         <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>222</v>
+        <v>193</v>
       </c>
       <c r="C42" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="D42" t="s">
         <v>50</v>
       </c>
       <c r="E42" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3890,19 +3162,19 @@
         <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>224</v>
+        <v>195</v>
       </c>
       <c r="C43" t="s">
-        <v>225</v>
+        <v>196</v>
       </c>
       <c r="D43" t="s">
         <v>54</v>
       </c>
       <c r="E43" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F43" t="s">
-        <v>226</v>
+        <v>197</v>
       </c>
       <c r="G43" t="n">
         <v>48</v>
@@ -3931,7 +3203,7 @@
         <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F44" t="s">
         <v>100</v>
@@ -3954,19 +3226,19 @@
         <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>227</v>
+        <v>198</v>
       </c>
       <c r="C45" t="s">
-        <v>225</v>
+        <v>196</v>
       </c>
       <c r="D45" t="s">
         <v>50</v>
       </c>
       <c r="E45" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F45" t="s">
-        <v>228</v>
+        <v>199</v>
       </c>
       <c r="G45" t="n">
         <v>39</v>
@@ -3986,7 +3258,7 @@
         <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>229</v>
+        <v>200</v>
       </c>
       <c r="C46" t="s">
         <v>105</v>
@@ -3995,10 +3267,10 @@
         <v>50</v>
       </c>
       <c r="E46" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F46" t="s">
-        <v>230</v>
+        <v>201</v>
       </c>
       <c r="G46" t="n">
         <v>31</v>
@@ -4018,7 +3290,7 @@
         <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>231</v>
+        <v>202</v>
       </c>
       <c r="C47" t="s">
         <v>99</v>
@@ -4027,7 +3299,7 @@
         <v>28</v>
       </c>
       <c r="E47" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="F47" t="s">
         <v>86</v>
@@ -4050,7 +3322,7 @@
         <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>232</v>
+        <v>203</v>
       </c>
       <c r="C48" t="s">
         <v>99</v>
@@ -4059,10 +3331,10 @@
         <v>50</v>
       </c>
       <c r="E48" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F48" t="s">
-        <v>233</v>
+        <v>204</v>
       </c>
       <c r="G48" t="n">
         <v>27</v>
@@ -4082,19 +3354,19 @@
         <v>97</v>
       </c>
       <c r="B49" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="C49" t="s">
-        <v>235</v>
+        <v>206</v>
       </c>
       <c r="D49" t="s">
         <v>50</v>
       </c>
       <c r="E49" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F49" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -4114,7 +3386,7 @@
         <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>237</v>
+        <v>208</v>
       </c>
       <c r="C50" t="s">
         <v>105</v>
@@ -4123,10 +3395,10 @@
         <v>50</v>
       </c>
       <c r="E50" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F50" t="s">
-        <v>238</v>
+        <v>209</v>
       </c>
       <c r="G50" t="n">
         <v>24</v>
@@ -4146,7 +3418,7 @@
         <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>239</v>
+        <v>210</v>
       </c>
       <c r="C51" t="s">
         <v>99</v>
@@ -4155,10 +3427,10 @@
         <v>50</v>
       </c>
       <c r="E51" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F51" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
       <c r="G51" t="n">
         <v>21</v>
@@ -4175,19 +3447,21 @@
     </row>
     <row r="52">
       <c r="A52"/>
-      <c r="B52"/>
+      <c r="B52" t="s">
+        <v>212</v>
+      </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="E52" t="s">
-        <v>195</v>
+        <v>109</v>
       </c>
       <c r="F52" t="s">
-        <v>82</v>
+        <v>213</v>
       </c>
       <c r="G52" t="n">
-        <v>186</v>
+        <v>3</v>
       </c>
       <c r="H52" t="s">
         <v>16</v>
@@ -4201,19 +3475,21 @@
     </row>
     <row r="53">
       <c r="A53"/>
-      <c r="B53"/>
+      <c r="B53" t="s">
+        <v>214</v>
+      </c>
       <c r="C53"/>
       <c r="D53" t="s">
-        <v>107</v>
+        <v>50</v>
       </c>
       <c r="E53" t="s">
-        <v>195</v>
+        <v>142</v>
       </c>
       <c r="F53" t="s">
-        <v>241</v>
+        <v>215</v>
       </c>
       <c r="G53" t="n">
-        <v>127</v>
+        <v>1</v>
       </c>
       <c r="H53" t="s">
         <v>16</v>
@@ -4227,209 +3503,29 @@
     </row>
     <row r="54">
       <c r="A54"/>
-      <c r="B54"/>
+      <c r="B54" t="s">
+        <v>216</v>
+      </c>
       <c r="C54"/>
       <c r="D54" t="s">
-        <v>107</v>
+        <v>41</v>
       </c>
       <c r="E54" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F54" t="s">
-        <v>242</v>
-      </c>
-      <c r="G54" t="n">
-        <v>74</v>
+        <v>217</v>
+      </c>
+      <c r="G54" t="e">
+        <v>#NUM!</v>
       </c>
       <c r="H54" t="s">
-        <v>16</v>
+        <v>218</v>
       </c>
       <c r="I54" t="s">
         <v>17</v>
       </c>
       <c r="J54" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55"/>
-      <c r="B55"/>
-      <c r="C55"/>
-      <c r="D55" t="s">
-        <v>107</v>
-      </c>
-      <c r="E55" t="s">
-        <v>195</v>
-      </c>
-      <c r="F55" t="s">
-        <v>241</v>
-      </c>
-      <c r="G55" t="n">
-        <v>74</v>
-      </c>
-      <c r="H55" t="s">
-        <v>16</v>
-      </c>
-      <c r="I55" t="s">
-        <v>17</v>
-      </c>
-      <c r="J55" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56"/>
-      <c r="B56"/>
-      <c r="C56"/>
-      <c r="D56" t="s">
-        <v>107</v>
-      </c>
-      <c r="E56" t="s">
-        <v>166</v>
-      </c>
-      <c r="F56" t="s">
-        <v>243</v>
-      </c>
-      <c r="G56" t="n">
-        <v>59</v>
-      </c>
-      <c r="H56" t="s">
-        <v>16</v>
-      </c>
-      <c r="I56" t="s">
-        <v>17</v>
-      </c>
-      <c r="J56" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57"/>
-      <c r="B57"/>
-      <c r="C57"/>
-      <c r="D57" t="s">
-        <v>107</v>
-      </c>
-      <c r="E57" t="s">
-        <v>139</v>
-      </c>
-      <c r="F57" t="s">
-        <v>112</v>
-      </c>
-      <c r="G57" t="n">
-        <v>53</v>
-      </c>
-      <c r="H57" t="s">
-        <v>16</v>
-      </c>
-      <c r="I57" t="s">
-        <v>17</v>
-      </c>
-      <c r="J57" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58"/>
-      <c r="B58"/>
-      <c r="C58"/>
-      <c r="D58" t="s">
-        <v>107</v>
-      </c>
-      <c r="E58" t="s">
-        <v>145</v>
-      </c>
-      <c r="F58" t="s">
-        <v>82</v>
-      </c>
-      <c r="G58" t="n">
-        <v>49</v>
-      </c>
-      <c r="H58" t="s">
-        <v>16</v>
-      </c>
-      <c r="I58" t="s">
-        <v>17</v>
-      </c>
-      <c r="J58" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59"/>
-      <c r="B59"/>
-      <c r="C59"/>
-      <c r="D59" t="s">
-        <v>107</v>
-      </c>
-      <c r="E59" t="s">
-        <v>139</v>
-      </c>
-      <c r="F59" t="s">
-        <v>244</v>
-      </c>
-      <c r="G59" t="n">
-        <v>48</v>
-      </c>
-      <c r="H59" t="s">
-        <v>16</v>
-      </c>
-      <c r="I59" t="s">
-        <v>17</v>
-      </c>
-      <c r="J59" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60"/>
-      <c r="B60"/>
-      <c r="C60"/>
-      <c r="D60" t="s">
-        <v>107</v>
-      </c>
-      <c r="E60" t="s">
-        <v>145</v>
-      </c>
-      <c r="F60" t="s">
-        <v>92</v>
-      </c>
-      <c r="G60" t="n">
-        <v>45</v>
-      </c>
-      <c r="H60" t="s">
-        <v>16</v>
-      </c>
-      <c r="I60" t="s">
-        <v>17</v>
-      </c>
-      <c r="J60" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61"/>
-      <c r="B61"/>
-      <c r="C61"/>
-      <c r="D61" t="s">
-        <v>107</v>
-      </c>
-      <c r="E61" t="s">
-        <v>139</v>
-      </c>
-      <c r="F61" t="s">
-        <v>128</v>
-      </c>
-      <c r="G61" t="n">
-        <v>43</v>
-      </c>
-      <c r="H61" t="s">
-        <v>16</v>
-      </c>
-      <c r="I61" t="s">
-        <v>17</v>
-      </c>
-      <c r="J61" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4458,7 +3554,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>245</v>
+        <v>219</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -4477,20 +3573,26 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2"/>
-      <c r="B2"/>
-      <c r="C2"/>
+      <c r="A2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" t="s">
+        <v>173</v>
+      </c>
       <c r="D2" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>195</v>
+        <v>109</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>174</v>
       </c>
       <c r="G2" t="n">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="H2" t="s">
         <v>16</v>
@@ -4504,25 +3606,25 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>157</v>
       </c>
       <c r="C3" t="s">
-        <v>202</v>
+        <v>65</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="F3" t="s">
-        <v>203</v>
+        <v>37</v>
       </c>
       <c r="G3" t="n">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H3" t="s">
         <v>16</v>
@@ -4539,22 +3641,22 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>118</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>159</v>
       </c>
       <c r="G4" t="n">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="H4" t="s">
         <v>16</v>
@@ -4568,51 +3670,57 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5" t="n">
+        <v>126</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
         <v>34</v>
       </c>
-      <c r="B5" t="s">
-        <v>188</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F5" t="s">
-        <v>189</v>
-      </c>
-      <c r="G5" t="n">
-        <v>144</v>
-      </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6"/>
-      <c r="B6"/>
-      <c r="C6"/>
+      <c r="B6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>195</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
-        <v>241</v>
+        <v>92</v>
       </c>
       <c r="G6" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="H6" t="s">
         <v>16</v>
@@ -4629,22 +3737,22 @@
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>177</v>
       </c>
       <c r="C7" t="s">
-        <v>205</v>
+        <v>178</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>195</v>
+        <v>109</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>179</v>
       </c>
       <c r="G7" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
@@ -4658,25 +3766,25 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>181</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="F8" t="s">
         <v>92</v>
       </c>
       <c r="G8" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H8" t="s">
         <v>16</v>
@@ -4693,22 +3801,22 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>206</v>
+        <v>182</v>
       </c>
       <c r="C9" t="s">
-        <v>207</v>
+        <v>183</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F9" t="s">
-        <v>208</v>
+        <v>110</v>
       </c>
       <c r="G9" t="n">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
@@ -4725,22 +3833,22 @@
         <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>209</v>
+        <v>184</v>
       </c>
       <c r="C10" t="s">
-        <v>210</v>
+        <v>185</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>186</v>
       </c>
       <c r="G10" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -4757,22 +3865,22 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>211</v>
+        <v>187</v>
       </c>
       <c r="C11" t="s">
-        <v>212</v>
+        <v>91</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
       <c r="F11" t="s">
-        <v>140</v>
+        <v>188</v>
       </c>
       <c r="G11" t="n">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@e36646b26fdacb2f10ca22fb6a846282dd7e1906 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -337,6 +337,18 @@
     <t xml:space="preserve">2025-12-20</t>
   </si>
   <si>
+    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolo - Hartonal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-18</t>
+  </si>
+  <si>
     <t xml:space="preserve">Riesgo</t>
   </si>
   <si>
@@ -629,15 +641,6 @@
   </si>
   <si>
     <t xml:space="preserve">2025-07-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bolo - Hartonal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-19</t>
   </si>
   <si>
     <t xml:space="preserve">MONASTIR_0436</t>
@@ -1802,6 +1805,38 @@
         <v>17</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" t="s">
+        <v>109</v>
+      </c>
+      <c r="F26" t="s">
+        <v>110</v>
+      </c>
+      <c r="G26" t="n">
+        <v>26</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1827,7 +1862,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1850,7 +1885,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1859,10 +1894,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G2" t="n">
         <v>74</v>
@@ -1882,19 +1917,19 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="G3" t="n">
         <v>70</v>
@@ -1914,19 +1949,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -1946,19 +1981,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G5" t="n">
         <v>63</v>
@@ -1978,19 +2013,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
         <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
@@ -2010,19 +2045,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D7" t="s">
         <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G7" t="n">
         <v>59</v>
@@ -2042,19 +2077,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D8" t="s">
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G8" t="n">
         <v>58</v>
@@ -2074,7 +2109,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2083,10 +2118,10 @@
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G9" t="n">
         <v>46</v>
@@ -2106,7 +2141,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
@@ -2115,7 +2150,7 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F10" t="s">
         <v>37</v>
@@ -2138,19 +2173,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F11" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G11" t="n">
         <v>34</v>
@@ -2167,22 +2202,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="G12" t="n">
         <v>62</v>
@@ -2199,22 +2234,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B13" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D13" t="s">
         <v>81</v>
       </c>
       <c r="E13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F13" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -2231,19 +2266,19 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D14" t="s">
         <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F14" t="s">
         <v>86</v>
@@ -2263,19 +2298,19 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B15" t="s">
+        <v>147</v>
+      </c>
+      <c r="C15" t="s">
         <v>143</v>
-      </c>
-      <c r="C15" t="s">
-        <v>139</v>
       </c>
       <c r="D15" t="s">
         <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F15" t="s">
         <v>37</v>
@@ -2295,22 +2330,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B16" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C16" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D16" t="s">
         <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F16" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G16" t="n">
         <v>6</v>
@@ -2327,22 +2362,22 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B17" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D17" t="s">
         <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F17" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -2359,22 +2394,22 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C18" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D18" t="s">
         <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F18" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -2391,22 +2426,22 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C19" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F19" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -2423,22 +2458,22 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B20" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C20" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D20" t="s">
         <v>85</v>
       </c>
       <c r="E20" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F20" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -2455,22 +2490,22 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D21" t="s">
         <v>85</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F21" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -2490,7 +2525,7 @@
         <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C22" t="s">
         <v>65</v>
@@ -2499,7 +2534,7 @@
         <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F22" t="s">
         <v>37</v>
@@ -2522,19 +2557,19 @@
         <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C23" t="s">
         <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="G23" t="n">
         <v>144</v>
@@ -2554,7 +2589,7 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C24" t="s">
         <v>65</v>
@@ -2563,7 +2598,7 @@
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F24" t="s">
         <v>92</v>
@@ -2586,19 +2621,19 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C25" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D25" t="s">
         <v>50</v>
       </c>
       <c r="E25" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F25" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G25" t="n">
         <v>100</v>
@@ -2627,7 +2662,7 @@
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F26" t="s">
         <v>37</v>
@@ -2650,16 +2685,16 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C27" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D27" t="s">
         <v>50</v>
       </c>
       <c r="E27" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F27" t="s">
         <v>58</v>
@@ -2691,7 +2726,7 @@
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F28" t="s">
         <v>46</v>
@@ -2714,7 +2749,7 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C29" t="s">
         <v>61</v>
@@ -2723,10 +2758,10 @@
         <v>50</v>
       </c>
       <c r="E29" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F29" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="G29" t="n">
         <v>67</v>
@@ -2746,7 +2781,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
         <v>65</v>
@@ -2755,10 +2790,10 @@
         <v>54</v>
       </c>
       <c r="E30" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F30" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="G30" t="n">
         <v>63</v>
@@ -2778,7 +2813,7 @@
         <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C31" t="s">
         <v>61</v>
@@ -2787,10 +2822,10 @@
         <v>54</v>
       </c>
       <c r="E31" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F31" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="G31" t="n">
         <v>63</v>
@@ -2810,19 +2845,19 @@
         <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C32" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F32" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G32" t="n">
         <v>156</v>
@@ -2842,16 +2877,16 @@
         <v>71</v>
       </c>
       <c r="B33" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C33" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F33" t="s">
         <v>82</v>
@@ -2874,19 +2909,19 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C34" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F34" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G34" t="n">
         <v>118</v>
@@ -2906,16 +2941,16 @@
         <v>71</v>
       </c>
       <c r="B35" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C35" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F35" t="s">
         <v>92</v>
@@ -2938,19 +2973,19 @@
         <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C36" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F36" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G36" t="n">
         <v>112</v>
@@ -2970,19 +3005,19 @@
         <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C37" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F37" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="G37" t="n">
         <v>106</v>
@@ -3002,7 +3037,7 @@
         <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C38" t="s">
         <v>91</v>
@@ -3011,10 +3046,10 @@
         <v>85</v>
       </c>
       <c r="E38" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F38" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="G38" t="n">
         <v>101</v>
@@ -3034,7 +3069,7 @@
         <v>71</v>
       </c>
       <c r="B39" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C39" t="s">
         <v>89</v>
@@ -3043,10 +3078,10 @@
         <v>28</v>
       </c>
       <c r="E39" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F39" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="G39" t="n">
         <v>98</v>
@@ -3066,7 +3101,7 @@
         <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C40" t="s">
         <v>94</v>
@@ -3075,10 +3110,10 @@
         <v>28</v>
       </c>
       <c r="E40" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F40" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="G40" t="n">
         <v>68</v>
@@ -3107,7 +3142,7 @@
         <v>28</v>
       </c>
       <c r="E41" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F41" t="s">
         <v>37</v>
@@ -3130,16 +3165,16 @@
         <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C42" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D42" t="s">
         <v>50</v>
       </c>
       <c r="E42" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3162,19 +3197,19 @@
         <v>97</v>
       </c>
       <c r="B43" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C43" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D43" t="s">
         <v>54</v>
       </c>
       <c r="E43" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F43" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="G43" t="n">
         <v>48</v>
@@ -3203,7 +3238,7 @@
         <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F44" t="s">
         <v>100</v>
@@ -3226,19 +3261,19 @@
         <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C45" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D45" t="s">
         <v>50</v>
       </c>
       <c r="E45" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F45" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="G45" t="n">
         <v>39</v>
@@ -3258,7 +3293,7 @@
         <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C46" t="s">
         <v>105</v>
@@ -3267,10 +3302,10 @@
         <v>50</v>
       </c>
       <c r="E46" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F46" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="G46" t="n">
         <v>31</v>
@@ -3290,7 +3325,7 @@
         <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C47" t="s">
         <v>99</v>
@@ -3299,7 +3334,7 @@
         <v>28</v>
       </c>
       <c r="E47" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F47" t="s">
         <v>86</v>
@@ -3322,7 +3357,7 @@
         <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C48" t="s">
         <v>99</v>
@@ -3331,10 +3366,10 @@
         <v>50</v>
       </c>
       <c r="E48" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F48" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G48" t="n">
         <v>27</v>
@@ -3354,19 +3389,19 @@
         <v>97</v>
       </c>
       <c r="B49" t="s">
-        <v>205</v>
+        <v>107</v>
       </c>
       <c r="C49" t="s">
-        <v>206</v>
+        <v>108</v>
       </c>
       <c r="D49" t="s">
         <v>50</v>
       </c>
       <c r="E49" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F49" t="s">
-        <v>207</v>
+        <v>109</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -3386,7 +3421,7 @@
         <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C50" t="s">
         <v>105</v>
@@ -3395,10 +3430,10 @@
         <v>50</v>
       </c>
       <c r="E50" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F50" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G50" t="n">
         <v>24</v>
@@ -3418,7 +3453,7 @@
         <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C51" t="s">
         <v>99</v>
@@ -3427,10 +3462,10 @@
         <v>50</v>
       </c>
       <c r="E51" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F51" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G51" t="n">
         <v>21</v>
@@ -3448,17 +3483,17 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
         <v>85</v>
       </c>
       <c r="E52" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F52" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
@@ -3476,17 +3511,17 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C53"/>
       <c r="D53" t="s">
         <v>50</v>
       </c>
       <c r="E53" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F53" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G53" t="n">
         <v>1</v>
@@ -3504,23 +3539,23 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C54"/>
       <c r="D54" t="s">
         <v>41</v>
       </c>
       <c r="E54" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F54" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G54" t="e">
         <v>#NUM!</v>
       </c>
       <c r="H54" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I54" t="s">
         <v>17</v>
@@ -3554,7 +3589,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -3577,19 +3612,19 @@
         <v>71</v>
       </c>
       <c r="B2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G2" t="n">
         <v>156</v>
@@ -3609,7 +3644,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C3" t="s">
         <v>65</v>
@@ -3618,7 +3653,7 @@
         <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F3" t="s">
         <v>37</v>
@@ -3641,19 +3676,19 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C4" t="s">
         <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="G4" t="n">
         <v>144</v>
@@ -3673,16 +3708,16 @@
         <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F5" t="s">
         <v>82</v>
@@ -3705,7 +3740,7 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C6" t="s">
         <v>65</v>
@@ -3714,7 +3749,7 @@
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F6" t="s">
         <v>92</v>
@@ -3737,19 +3772,19 @@
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F7" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G7" t="n">
         <v>118</v>
@@ -3769,16 +3804,16 @@
         <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D8" t="s">
         <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F8" t="s">
         <v>92</v>
@@ -3801,19 +3836,19 @@
         <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C9" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G9" t="n">
         <v>112</v>
@@ -3833,19 +3868,19 @@
         <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C10" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F10" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="G10" t="n">
         <v>106</v>
@@ -3865,7 +3900,7 @@
         <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C11" t="s">
         <v>91</v>
@@ -3874,10 +3909,10 @@
         <v>85</v>
       </c>
       <c r="E11" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F11" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="G11" t="n">
         <v>101</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@437f8e7896218fba120c210f8ca465eff5834670 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -671,9 +671,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sin Eventos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visita Preventiva</t>
   </si>
   <si>
     <t xml:space="preserve">Nivel</t>
@@ -3555,7 +3552,7 @@
         <v>#NUM!</v>
       </c>
       <c r="H54" t="s">
-        <v>219</v>
+        <v>16</v>
       </c>
       <c r="I54" t="s">
         <v>17</v>
@@ -3589,7 +3586,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@9fe499f1e4f30e1fadc569ae6a7b2d431bd1337e 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -118,403 +118,424 @@
     <t xml:space="preserve">2026-06-09</t>
   </si>
   <si>
+    <t xml:space="preserve">REGINA 3_0682</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENTRAL CASTILLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Colombiana_17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arenal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caideal_78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-20</t>
+  </si>
+  <si>
     <t xml:space="preserve">Florida</t>
   </si>
   <si>
+    <t xml:space="preserve">EL REFUGIO 1, 2 Y 3_010139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chococito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INCAUCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Casilda_274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Pedregal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IND. DORIS_0453</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio de los Caballeros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA INDUSTRIA_752</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA CABAÑA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PISAMOS_0768</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REY 2_0784</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Diana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BELGICA_0780</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Remolino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOS RANCHOS_0466</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palmira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Chica Gaviria_272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caucaseco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAN PABLO TUMACO_011948</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guanabanal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-05-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HERRAGRICOLA_2493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palmaseca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PICHICHI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRANSITO CENTRAL TUMACO_081369</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Herradura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROVIDENCIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANTA ROSA_347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tienda Nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORIENTE_362</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guayabal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JOSEPILLA_359</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obando</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pradera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL ARADO_460</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Floresta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Guaira_116</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Tupia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL CUBO 1_0570</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Granja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolo - Hartonal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riesgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cofre_18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MITIGADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-09-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potrero de PA rraga_36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-09-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Arenal_48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA I_000204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARIA LUISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARGARITAS_0448</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Joaquin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabuyal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHONDULAR_940</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-08-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Palmar_88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA GUACA III_000207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Cerrito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brisuelas_302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Helena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVACION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-02-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENOVA_2281</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-12-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL ALBION_080402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAJO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA HOLANDA_080355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAMARIA_080104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Placer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-01-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL PLACER_080489</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024-11-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURIN_080435</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-03-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFLEJO_305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-08-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROVIDENCIA_080101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-05-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA PAZ_080102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-07-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIERRA GRATA_0703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGENIO_000502</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-01-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Retiro_384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA ESTRELLA_0725</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santa Rosa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Arauca_32</t>
   </si>
   <si>
     <t xml:space="preserve">Tarragona</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL REFUGIO 1, 2 Y 3_010139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chococito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INCAUCA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Casilda_274</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Pedregal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IND. DORIS_0453</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Antonio de los Caballeros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CENTRAL CASTILLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA INDUSTRIA_752</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA CABAÑA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PISAMOS_0768</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REY 2_0784</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Diana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BELGICA_0780</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Remolino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOS RANCHOS_0466</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Palmira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Chica Gaviria_272</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caucaseco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAN PABLO TUMACO_011948</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guanabanal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HERRAGRICOLA_2493</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Palmaseca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PICHICHI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRANSITO CENTRAL TUMACO_081369</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Herradura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROVIDENCIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SANTA ROSA_347</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tienda Nueva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORIENTE_362</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guayabal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JOSEPILLA_359</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obando</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pradera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL ARADO_460</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Floresta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Guaira_116</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Tupia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL CUBO 1_0570</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Granja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PORVENIR LOPEZ_0260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bolo - Hartonal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riesgo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cofre_18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MITIGADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-09-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potrero de PA rraga_36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arenal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Arenal_48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRITICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA I_000204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARIA LUISA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MARGARITAS_0448</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Joaquin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARGENTINA DIES Y LOME_C38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabuyal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL COFRE CASASFRANCO_010250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHONDULAR_940</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-08-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Palmar_88</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA GUACA III_000207</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-01-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Cerrito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brisuelas_302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Helena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVACION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GENOVA_2281</t>
-  </si>
-  <si>
-    <t xml:space="preserve">San Antonio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-12-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL ALBION_080402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BAJO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA HOLANDA_080355</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMARIA_080104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Placer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-01-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL PLACER_080489</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TURIN_080435</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-03-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFLEJO_305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-08-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROVIDENCIA_080101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2020-05-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA PAZ_080102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-07-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIERRA GRATA_0703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INGENIO_000502</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Retiro_384</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA ESTRELLA_0725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santa Rosa</t>
   </si>
   <si>
     <t xml:space="preserve">SAN RAFAEL H._0687</t>
@@ -1196,25 +1217,25 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
         <v>35</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>37</v>
       </c>
-      <c r="F7" t="s">
-        <v>38</v>
-      </c>
       <c r="G7" t="n">
-        <v>98</v>
+        <v>33</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
@@ -1228,25 +1249,25 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G8" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="H8" t="s">
         <v>16</v>
@@ -1260,25 +1281,25 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G9" t="n">
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
@@ -1292,25 +1313,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
         <v>48</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>49</v>
       </c>
-      <c r="D10" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" t="s">
-        <v>52</v>
-      </c>
       <c r="G10" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -1324,25 +1345,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" t="s">
         <v>53</v>
       </c>
-      <c r="C11" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" t="s">
-        <v>56</v>
-      </c>
       <c r="G11" t="n">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -1356,25 +1377,25 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
         <v>57</v>
       </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" t="s">
-        <v>58</v>
-      </c>
-      <c r="F12" t="s">
-        <v>59</v>
-      </c>
       <c r="G12" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -1388,25 +1409,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
         <v>60</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>61</v>
       </c>
-      <c r="D13" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" t="s">
-        <v>63</v>
-      </c>
       <c r="G13" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -1420,25 +1441,25 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
         <v>64</v>
       </c>
-      <c r="C14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" t="s">
-        <v>67</v>
-      </c>
       <c r="G14" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -1452,25 +1473,25 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" t="s">
         <v>68</v>
       </c>
-      <c r="C15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" t="s">
-        <v>70</v>
-      </c>
       <c r="G15" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -1484,25 +1505,25 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" t="s">
         <v>71</v>
       </c>
-      <c r="B16" t="s">
+      <c r="F16" t="s">
         <v>72</v>
       </c>
-      <c r="C16" t="s">
-        <v>73</v>
-      </c>
-      <c r="D16" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" t="s">
-        <v>74</v>
-      </c>
-      <c r="F16" t="s">
-        <v>47</v>
-      </c>
       <c r="G16" t="n">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
@@ -1516,25 +1537,25 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" t="s">
         <v>75</v>
       </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" t="s">
-        <v>78</v>
-      </c>
       <c r="G17" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="H17" t="s">
         <v>16</v>
@@ -1548,25 +1569,25 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
         <v>79</v>
       </c>
-      <c r="C18" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" t="s">
-        <v>81</v>
-      </c>
-      <c r="E18" t="s">
-        <v>82</v>
-      </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G18" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
@@ -1580,25 +1601,25 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" t="s">
         <v>83</v>
       </c>
-      <c r="C19" t="s">
-        <v>84</v>
-      </c>
-      <c r="D19" t="s">
-        <v>85</v>
-      </c>
-      <c r="E19" t="s">
-        <v>86</v>
-      </c>
-      <c r="F19" t="s">
-        <v>87</v>
-      </c>
       <c r="G19" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H19" t="s">
         <v>16</v>
@@ -1612,25 +1633,25 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="E20" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G20" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="H20" t="s">
         <v>16</v>
@@ -1644,25 +1665,25 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D21" t="s">
         <v>90</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>91</v>
       </c>
-      <c r="D21" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>92</v>
       </c>
-      <c r="F21" t="s">
-        <v>33</v>
-      </c>
       <c r="G21" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H21" t="s">
         <v>16</v>
@@ -1676,7 +1697,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
         <v>93</v>
@@ -1691,10 +1712,10 @@
         <v>95</v>
       </c>
       <c r="F22" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="G22" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="H22" t="s">
         <v>16</v>
@@ -1708,25 +1729,25 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" t="s">
         <v>97</v>
-      </c>
-      <c r="B23" t="s">
-        <v>98</v>
-      </c>
-      <c r="C23" t="s">
-        <v>99</v>
       </c>
       <c r="D23" t="s">
         <v>28</v>
       </c>
       <c r="E23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F23" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="G23" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="H23" t="s">
         <v>16</v>
@@ -1740,25 +1761,25 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" t="s">
         <v>101</v>
       </c>
-      <c r="C24" t="s">
+      <c r="F24" t="s">
         <v>102</v>
       </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" t="s">
-        <v>103</v>
-      </c>
-      <c r="F24" t="s">
-        <v>67</v>
-      </c>
       <c r="G24" t="n">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="H24" t="s">
         <v>16</v>
@@ -1772,7 +1793,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B25" t="s">
         <v>104</v>
@@ -1781,16 +1802,16 @@
         <v>105</v>
       </c>
       <c r="D25" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="E25" t="s">
         <v>106</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="G25" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="H25" t="s">
         <v>16</v>
@@ -1804,7 +1825,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B26" t="s">
         <v>107</v>
@@ -1813,24 +1834,88 @@
         <v>108</v>
       </c>
       <c r="D26" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
         <v>109</v>
       </c>
       <c r="F26" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" t="n">
+        <v>16</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" t="s">
         <v>110</v>
       </c>
-      <c r="G26" t="n">
+      <c r="C27" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" t="s">
+        <v>75</v>
+      </c>
+      <c r="G27" t="n">
+        <v>14</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" t="s">
+        <v>114</v>
+      </c>
+      <c r="D28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" t="s">
+        <v>115</v>
+      </c>
+      <c r="F28" t="s">
+        <v>116</v>
+      </c>
+      <c r="G28" t="n">
         <v>26</v>
       </c>
-      <c r="H26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" t="s">
-        <v>17</v>
-      </c>
-      <c r="J26" t="s">
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1859,7 +1944,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1882,7 +1967,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1891,10 +1976,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F2" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G2" t="n">
         <v>74</v>
@@ -1914,19 +1999,19 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="G3" t="n">
         <v>70</v>
@@ -1946,19 +2031,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -1978,19 +2063,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="G5" t="n">
         <v>63</v>
@@ -2010,19 +2095,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
         <v>124</v>
       </c>
-      <c r="C6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" t="s">
-        <v>119</v>
-      </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
@@ -2042,19 +2127,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="G7" t="n">
         <v>59</v>
@@ -2074,19 +2159,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F8" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="G8" t="n">
         <v>58</v>
@@ -2106,7 +2191,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2115,10 +2200,10 @@
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="G9" t="n">
         <v>46</v>
@@ -2138,7 +2223,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
@@ -2147,10 +2232,10 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G10" t="n">
         <v>45</v>
@@ -2170,19 +2255,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="G11" t="n">
         <v>34</v>
@@ -2199,22 +2284,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B12" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C12" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="G12" t="n">
         <v>62</v>
@@ -2231,22 +2316,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E13" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F13" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -2263,22 +2348,22 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C14" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D14" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E14" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G14" t="n">
         <v>10</v>
@@ -2295,22 +2380,22 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C15" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D15" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F15" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G15" t="n">
         <v>7</v>
@@ -2327,22 +2412,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C16" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G16" t="n">
         <v>6</v>
@@ -2359,22 +2444,22 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B17" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E17" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F17" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -2391,22 +2476,22 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B18" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C18" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D18" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F18" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -2423,22 +2508,22 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B19" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C19" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F19" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -2455,22 +2540,22 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="C20" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F20" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -2487,22 +2572,22 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B21" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C21" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F21" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -2519,22 +2604,22 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B22" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E22" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F22" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G22" t="n">
         <v>154</v>
@@ -2551,22 +2636,22 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F23" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G23" t="n">
         <v>144</v>
@@ -2583,22 +2668,22 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D24" t="s">
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G24" t="n">
         <v>119</v>
@@ -2615,22 +2700,22 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B25" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C25" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D25" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F25" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G25" t="n">
         <v>100</v>
@@ -2647,22 +2732,22 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>173</v>
       </c>
       <c r="D26" t="s">
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F26" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G26" t="n">
         <v>98</v>
@@ -2679,22 +2764,22 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C27" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D27" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E27" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F27" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G27" t="n">
         <v>82</v>
@@ -2711,22 +2796,22 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G28" t="n">
         <v>79</v>
@@ -2743,22 +2828,22 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B29" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E29" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F29" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="G29" t="n">
         <v>67</v>
@@ -2775,22 +2860,22 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D30" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E30" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F30" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="G30" t="n">
         <v>63</v>
@@ -2807,22 +2892,22 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B31" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E31" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="F31" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="G31" t="n">
         <v>63</v>
@@ -2839,22 +2924,22 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C32" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F32" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="G32" t="n">
         <v>156</v>
@@ -2871,22 +2956,22 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C33" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F33" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G33" t="n">
         <v>126</v>
@@ -2903,22 +2988,22 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C34" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F34" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="G34" t="n">
         <v>118</v>
@@ -2935,22 +3020,22 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C35" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F35" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G35" t="n">
         <v>117</v>
@@ -2967,22 +3052,22 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C36" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F36" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G36" t="n">
         <v>112</v>
@@ -2999,22 +3084,22 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C37" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F37" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="G37" t="n">
         <v>106</v>
@@ -3031,22 +3116,22 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C38" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F38" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="G38" t="n">
         <v>101</v>
@@ -3063,22 +3148,22 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C39" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D39" t="s">
         <v>28</v>
       </c>
       <c r="E39" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F39" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="G39" t="n">
         <v>98</v>
@@ -3095,22 +3180,22 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C40" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D40" t="s">
         <v>28</v>
       </c>
       <c r="E40" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F40" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="G40" t="n">
         <v>68</v>
@@ -3127,22 +3212,22 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C41" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
         <v>28</v>
       </c>
       <c r="E41" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F41" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G41" t="n">
         <v>57</v>
@@ -3159,19 +3244,19 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B42" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C42" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="D42" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E42" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3191,22 +3276,22 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B43" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C43" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="D43" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E43" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F43" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="G43" t="n">
         <v>48</v>
@@ -3223,22 +3308,22 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B44" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C44" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D44" t="s">
         <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F44" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="G44" t="n">
         <v>47</v>
@@ -3255,22 +3340,22 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B45" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C45" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="D45" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E45" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F45" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="G45" t="n">
         <v>39</v>
@@ -3287,22 +3372,22 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C46" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D46" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E46" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F46" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="G46" t="n">
         <v>31</v>
@@ -3319,22 +3404,22 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B47" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C47" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
       </c>
       <c r="E47" t="s">
-        <v>169</v>
+        <v>124</v>
       </c>
       <c r="F47" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G47" t="n">
         <v>31</v>
@@ -3351,22 +3436,22 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B48" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C48" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D48" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E48" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F48" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="G48" t="n">
         <v>27</v>
@@ -3383,22 +3468,22 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C49" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D49" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E49" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F49" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -3415,22 +3500,22 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B50" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C50" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E50" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F50" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="G50" t="n">
         <v>24</v>
@@ -3447,22 +3532,22 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B51" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D51" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E51" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F51" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="G51" t="n">
         <v>21</v>
@@ -3480,17 +3565,17 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E52" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F52" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
@@ -3508,17 +3593,17 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C53"/>
       <c r="D53" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E53" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F53" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="G53" t="n">
         <v>1</v>
@@ -3536,17 +3621,17 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C54"/>
       <c r="D54" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E54" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F54" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="G54" t="e">
         <v>#NUM!</v>
@@ -3586,7 +3671,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -3606,22 +3691,22 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F2" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="G2" t="n">
         <v>156</v>
@@ -3638,22 +3723,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="G3" t="n">
         <v>154</v>
@@ -3670,22 +3755,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F4" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G4" t="n">
         <v>144</v>
@@ -3702,22 +3787,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C5" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G5" t="n">
         <v>126</v>
@@ -3734,22 +3819,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G6" t="n">
         <v>119</v>
@@ -3766,22 +3851,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C7" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="G7" t="n">
         <v>118</v>
@@ -3798,22 +3883,22 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C8" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D8" t="s">
         <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G8" t="n">
         <v>117</v>
@@ -3830,22 +3915,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C9" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G9" t="n">
         <v>112</v>
@@ -3862,22 +3947,22 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C10" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F10" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="G10" t="n">
         <v>106</v>
@@ -3894,22 +3979,22 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="F11" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="G11" t="n">
         <v>101</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ secasor/SATICA-V2@e2a6b5cc4f515e38c839c24fac5f502fe660f0c2 🚀
</commit_message>
<xml_diff>
--- a/data_master/SATICA_Seguimiento_latest.xlsx
+++ b/data_master/SATICA_Seguimiento_latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="229">
   <si>
     <t xml:space="preserve">Municipio</t>
   </si>
@@ -148,6 +148,12 @@
     <t xml:space="preserve">2026-06-20</t>
   </si>
   <si>
+    <t xml:space="preserve">El Palmar_88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-25</t>
+  </si>
+  <si>
     <t xml:space="preserve">Florida</t>
   </si>
   <si>
@@ -301,9 +307,6 @@
     <t xml:space="preserve">Tienda Nueva</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-04-25</t>
-  </si>
-  <si>
     <t xml:space="preserve">ORIENTE_362</t>
   </si>
   <si>
@@ -325,6 +328,15 @@
     <t xml:space="preserve">2026-06-14</t>
   </si>
   <si>
+    <t xml:space="preserve">OLGA_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-03</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pradera</t>
   </si>
   <si>
@@ -433,9 +445,6 @@
     <t xml:space="preserve">2025-08-02</t>
   </si>
   <si>
-    <t xml:space="preserve">El Palmar_88</t>
-  </si>
-  <si>
     <t xml:space="preserve">LA GUACA III_000207</t>
   </si>
   <si>
@@ -611,9 +620,6 @@
   </si>
   <si>
     <t xml:space="preserve">ESPERANZA INESA_081363</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-03</t>
   </si>
   <si>
     <t xml:space="preserve">CABAA'A_001</t>
@@ -1313,25 +1319,25 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
         <v>44</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
         <v>45</v>
       </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" t="s">
-        <v>48</v>
-      </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G10" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -1345,25 +1351,25 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" t="s">
         <v>50</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>51</v>
       </c>
-      <c r="D11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" t="s">
-        <v>53</v>
-      </c>
       <c r="G11" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -1377,25 +1383,25 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
         <v>54</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
         <v>55</v>
       </c>
-      <c r="D12" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" t="s">
-        <v>57</v>
-      </c>
       <c r="G12" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -1409,25 +1415,25 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="F13" t="s">
         <v>59</v>
       </c>
-      <c r="E13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F13" t="s">
-        <v>61</v>
-      </c>
       <c r="G13" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -1441,25 +1447,25 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
         <v>62</v>
       </c>
-      <c r="C14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>63</v>
       </c>
-      <c r="F14" t="s">
-        <v>64</v>
-      </c>
       <c r="G14" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -1473,25 +1479,25 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
         <v>35</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -1505,25 +1511,25 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
         <v>35</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G16" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
@@ -1537,25 +1543,25 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D17" t="s">
         <v>35</v>
       </c>
       <c r="E17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" t="s">
         <v>74</v>
       </c>
-      <c r="F17" t="s">
-        <v>75</v>
-      </c>
       <c r="G17" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="H17" t="s">
         <v>16</v>
@@ -1569,25 +1575,25 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" t="s">
         <v>76</v>
       </c>
-      <c r="B18" t="s">
+      <c r="F18" t="s">
         <v>77</v>
       </c>
-      <c r="C18" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>79</v>
-      </c>
-      <c r="F18" t="s">
-        <v>53</v>
-      </c>
       <c r="G18" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
@@ -1601,25 +1607,25 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" t="s">
         <v>80</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
         <v>81</v>
       </c>
-      <c r="D19" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" t="s">
-        <v>82</v>
-      </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="G19" t="n">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="H19" t="s">
         <v>16</v>
@@ -1633,25 +1639,25 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" t="s">
         <v>84</v>
       </c>
-      <c r="C20" t="s">
+      <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="D20" t="s">
-        <v>86</v>
-      </c>
-      <c r="E20" t="s">
-        <v>87</v>
-      </c>
-      <c r="F20" t="s">
-        <v>57</v>
-      </c>
       <c r="G20" t="n">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="H20" t="s">
         <v>16</v>
@@ -1665,25 +1671,25 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" t="s">
         <v>88</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>89</v>
       </c>
-      <c r="D21" t="s">
-        <v>90</v>
-      </c>
-      <c r="E21" t="s">
-        <v>91</v>
-      </c>
       <c r="F21" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="G21" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="H21" t="s">
         <v>16</v>
@@ -1697,22 +1703,22 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" t="s">
         <v>93</v>
       </c>
-      <c r="C22" t="s">
+      <c r="F22" t="s">
         <v>94</v>
-      </c>
-      <c r="D22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22" t="s">
-        <v>95</v>
-      </c>
-      <c r="F22" t="s">
-        <v>61</v>
       </c>
       <c r="G22" t="n">
         <v>57</v>
@@ -1729,25 +1735,25 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" t="s">
         <v>96</v>
-      </c>
-      <c r="C23" t="s">
-        <v>97</v>
       </c>
       <c r="D23" t="s">
         <v>28</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="F23" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="G23" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H23" t="s">
         <v>16</v>
@@ -1761,25 +1767,25 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D24" t="s">
         <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F24" t="s">
-        <v>102</v>
+        <v>33</v>
       </c>
       <c r="G24" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="H24" t="s">
         <v>16</v>
@@ -1793,25 +1799,25 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D25" t="s">
         <v>28</v>
       </c>
       <c r="E25" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>103</v>
       </c>
       <c r="G25" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H25" t="s">
         <v>16</v>
@@ -1825,25 +1831,25 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D26" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F26" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="G26" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="H26" t="s">
         <v>16</v>
@@ -1857,25 +1863,25 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" t="s">
+        <v>109</v>
+      </c>
+      <c r="D27" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" t="s">
         <v>110</v>
       </c>
-      <c r="C27" t="s">
-        <v>111</v>
-      </c>
-      <c r="D27" t="s">
-        <v>35</v>
-      </c>
-      <c r="E27" t="s">
-        <v>112</v>
-      </c>
       <c r="F27" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="G27" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="H27" t="s">
         <v>16</v>
@@ -1889,33 +1895,97 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" t="s">
+        <v>112</v>
+      </c>
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" t="s">
         <v>113</v>
       </c>
-      <c r="C28" t="s">
+      <c r="F28" t="s">
+        <v>74</v>
+      </c>
+      <c r="G28" t="n">
+        <v>16</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" t="s">
         <v>114</v>
       </c>
-      <c r="D28" t="s">
+      <c r="C29" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" t="s">
         <v>35</v>
       </c>
-      <c r="E28" t="s">
-        <v>115</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="E29" t="s">
         <v>116</v>
       </c>
-      <c r="G28" t="n">
+      <c r="F29" t="s">
+        <v>77</v>
+      </c>
+      <c r="G29" t="n">
+        <v>14</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" t="s">
+        <v>17</v>
+      </c>
+      <c r="J29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>107</v>
+      </c>
+      <c r="B30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" t="s">
+        <v>119</v>
+      </c>
+      <c r="F30" t="s">
+        <v>120</v>
+      </c>
+      <c r="G30" t="n">
         <v>26</v>
       </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" t="s">
-        <v>17</v>
-      </c>
-      <c r="J28" t="s">
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1944,7 +2014,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1967,7 +2037,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -1976,10 +2046,10 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G2" t="n">
         <v>74</v>
@@ -1999,7 +2069,7 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
@@ -2008,10 +2078,10 @@
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G3" t="n">
         <v>70</v>
@@ -2031,7 +2101,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C4" t="s">
         <v>39</v>
@@ -2040,10 +2110,10 @@
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G4" t="n">
         <v>67</v>
@@ -2063,19 +2133,19 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
         <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G5" t="n">
         <v>63</v>
@@ -2095,19 +2165,19 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D6" t="s">
         <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
@@ -2127,19 +2197,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G7" t="n">
         <v>59</v>
@@ -2159,19 +2229,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F8" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G8" t="n">
         <v>58</v>
@@ -2191,7 +2261,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2200,10 +2270,10 @@
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G9" t="n">
         <v>46</v>
@@ -2223,7 +2293,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
@@ -2232,10 +2302,10 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F10" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G10" t="n">
         <v>45</v>
@@ -2255,19 +2325,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G11" t="n">
         <v>34</v>
@@ -2284,22 +2354,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G12" t="n">
         <v>62</v>
@@ -2316,22 +2386,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" t="s">
         <v>148</v>
       </c>
-      <c r="D13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" t="s">
-        <v>145</v>
-      </c>
       <c r="F13" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G13" t="n">
         <v>25</v>
@@ -2348,22 +2418,22 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B14" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G14" t="n">
         <v>10</v>
@@ -2380,22 +2450,22 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F15" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G15" t="n">
         <v>7</v>
@@ -2412,22 +2482,22 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C16" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F16" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G16" t="n">
         <v>6</v>
@@ -2444,22 +2514,22 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B17" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F17" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -2476,22 +2546,22 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B18" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -2508,22 +2578,22 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B19" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F19" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -2540,22 +2610,22 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B20" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C20" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E20" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -2572,22 +2642,22 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B21" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C21" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E21" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -2604,22 +2674,22 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D22" t="s">
         <v>35</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G22" t="n">
         <v>154</v>
@@ -2636,22 +2706,22 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E23" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F23" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G23" t="n">
         <v>144</v>
@@ -2668,22 +2738,22 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D24" t="s">
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F24" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G24" t="n">
         <v>119</v>
@@ -2700,22 +2770,22 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B25" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C25" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D25" t="s">
         <v>35</v>
       </c>
       <c r="E25" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F25" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G25" t="n">
         <v>100</v>
@@ -2732,22 +2802,22 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C26" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D26" t="s">
         <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G26" t="n">
         <v>98</v>
@@ -2764,22 +2834,22 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B27" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C27" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D27" t="s">
         <v>35</v>
       </c>
       <c r="E27" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F27" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G27" t="n">
         <v>82</v>
@@ -2796,22 +2866,22 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F28" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G28" t="n">
         <v>79</v>
@@ -2828,22 +2898,22 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B29" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
         <v>35</v>
       </c>
       <c r="E29" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F29" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G29" t="n">
         <v>67</v>
@@ -2860,22 +2930,22 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B30" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G30" t="n">
         <v>63</v>
@@ -2892,22 +2962,22 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E31" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F31" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="G31" t="n">
         <v>63</v>
@@ -2924,22 +2994,22 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C32" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
       </c>
       <c r="E32" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F32" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G32" t="n">
         <v>156</v>
@@ -2956,22 +3026,22 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B33" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C33" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
       </c>
       <c r="E33" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G33" t="n">
         <v>126</v>
@@ -2988,22 +3058,22 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B34" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C34" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
       </c>
       <c r="E34" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F34" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G34" t="n">
         <v>118</v>
@@ -3020,22 +3090,22 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B35" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C35" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
       </c>
       <c r="E35" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F35" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G35" t="n">
         <v>117</v>
@@ -3052,22 +3122,22 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B36" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C36" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
       </c>
       <c r="E36" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F36" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G36" t="n">
         <v>112</v>
@@ -3084,22 +3154,22 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B37" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C37" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F37" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G37" t="n">
         <v>106</v>
@@ -3116,22 +3186,22 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C38" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E38" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F38" t="s">
-        <v>199</v>
+        <v>106</v>
       </c>
       <c r="G38" t="n">
         <v>101</v>
@@ -3148,22 +3218,22 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C39" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D39" t="s">
         <v>28</v>
       </c>
       <c r="E39" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F39" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G39" t="n">
         <v>98</v>
@@ -3180,22 +3250,22 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B40" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D40" t="s">
         <v>28</v>
       </c>
       <c r="E40" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F40" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G40" t="n">
         <v>68</v>
@@ -3212,22 +3282,22 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D41" t="s">
         <v>28</v>
       </c>
       <c r="E41" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F41" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G41" t="n">
         <v>57</v>
@@ -3244,19 +3314,19 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B42" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C42" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D42" t="s">
         <v>35</v>
       </c>
       <c r="E42" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3276,22 +3346,22 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B43" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C43" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D43" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E43" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F43" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G43" t="n">
         <v>48</v>
@@ -3308,22 +3378,22 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B44" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C44" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D44" t="s">
         <v>28</v>
       </c>
       <c r="E44" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F44" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G44" t="n">
         <v>47</v>
@@ -3340,22 +3410,22 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B45" t="s">
+        <v>211</v>
+      </c>
+      <c r="C45" t="s">
         <v>209</v>
-      </c>
-      <c r="C45" t="s">
-        <v>207</v>
       </c>
       <c r="D45" t="s">
         <v>35</v>
       </c>
       <c r="E45" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F45" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G45" t="n">
         <v>39</v>
@@ -3372,22 +3442,22 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B46" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D46" t="s">
         <v>35</v>
       </c>
       <c r="E46" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F46" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G46" t="n">
         <v>31</v>
@@ -3404,22 +3474,22 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B47" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C47" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
       </c>
       <c r="E47" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F47" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G47" t="n">
         <v>31</v>
@@ -3436,22 +3506,22 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B48" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C48" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D48" t="s">
         <v>35</v>
       </c>
       <c r="E48" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F48" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G48" t="n">
         <v>27</v>
@@ -3468,22 +3538,22 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C49" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D49" t="s">
         <v>35</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F49" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G49" t="n">
         <v>26</v>
@@ -3500,22 +3570,22 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B50" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C50" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D50" t="s">
         <v>35</v>
       </c>
       <c r="E50" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F50" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G50" t="n">
         <v>24</v>
@@ -3532,22 +3602,22 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B51" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C51" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D51" t="s">
         <v>35</v>
       </c>
       <c r="E51" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F51" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G51" t="n">
         <v>21</v>
@@ -3565,17 +3635,17 @@
     <row r="52">
       <c r="A52"/>
       <c r="B52" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C52"/>
       <c r="D52" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E52" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F52" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G52" t="n">
         <v>3</v>
@@ -3593,17 +3663,17 @@
     <row r="53">
       <c r="A53"/>
       <c r="B53" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C53"/>
       <c r="D53" t="s">
         <v>35</v>
       </c>
       <c r="E53" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F53" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G53" t="n">
         <v>1</v>
@@ -3621,17 +3691,17 @@
     <row r="54">
       <c r="A54"/>
       <c r="B54" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C54"/>
       <c r="D54" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E54" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F54" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G54" t="e">
         <v>#NUM!</v>
@@ -3671,7 +3741,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -3691,22 +3761,22 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G2" t="n">
         <v>156</v>
@@ -3723,22 +3793,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
         <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F3" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="G3" t="n">
         <v>154</v>
@@ -3755,22 +3825,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G4" t="n">
         <v>144</v>
@@ -3787,22 +3857,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G5" t="n">
         <v>126</v>
@@ -3819,22 +3889,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G6" t="n">
         <v>119</v>
@@ -3851,22 +3921,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G7" t="n">
         <v>118</v>
@@ -3883,22 +3953,22 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D8" t="s">
         <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G8" t="n">
         <v>117</v>
@@ -3915,22 +3985,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C9" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F9" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G9" t="n">
         <v>112</v>
@@ -3947,22 +4017,22 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C10" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F10" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G10" t="n">
         <v>106</v>
@@ -3979,22 +4049,22 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E11" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F11" t="s">
-        <v>199</v>
+        <v>106</v>
       </c>
       <c r="G11" t="n">
         <v>101</v>

</xml_diff>